<commit_message>
One of the coauthors had an updated bee species list following verification. Committing changes made following the addition of these species to the presence absence data and rerunning the regional species pool
</commit_message>
<xml_diff>
--- a/bcomm_23.localanalysis.xlsx
+++ b/bcomm_23.localanalysis.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ohio_Beesnew\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ohio_Bees\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{21066EF6-3234-4B1C-B5D0-75B8C33760B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20EAD675-4546-458C-B90B-4C06359117EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-26595" yWindow="3285" windowWidth="14400" windowHeight="8175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bcomm_23.localanalysis" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1345,7 +1358,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1482,7 +1495,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1662,6 +1675,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1823,11 +1842,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1887,9 +1907,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1927,7 +1947,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2033,7 +2053,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2175,14 +2195,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:MY72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -57064,7 +57084,7 @@
       <c r="DE51">
         <v>0</v>
       </c>
-      <c r="DF51">
+      <c r="DF51" s="2">
         <v>1</v>
       </c>
       <c r="DG51">
@@ -58107,8 +58127,8 @@
       <c r="CO52">
         <v>0</v>
       </c>
-      <c r="CP52">
-        <v>0</v>
+      <c r="CP52" s="2">
+        <v>1</v>
       </c>
       <c r="CQ52">
         <v>0</v>
@@ -58116,8 +58136,8 @@
       <c r="CR52">
         <v>0</v>
       </c>
-      <c r="CS52">
-        <v>0</v>
+      <c r="CS52" s="2">
+        <v>1</v>
       </c>
       <c r="CT52">
         <v>0</v>
@@ -58140,8 +58160,8 @@
       <c r="CZ52">
         <v>0</v>
       </c>
-      <c r="DA52">
-        <v>0</v>
+      <c r="DA52" s="2">
+        <v>1</v>
       </c>
       <c r="DB52">
         <v>0</v>
@@ -58155,11 +58175,11 @@
       <c r="DE52">
         <v>0</v>
       </c>
-      <c r="DF52">
-        <v>0</v>
-      </c>
-      <c r="DG52">
-        <v>0</v>
+      <c r="DF52" s="2">
+        <v>1</v>
+      </c>
+      <c r="DG52" s="2">
+        <v>1</v>
       </c>
       <c r="DH52">
         <v>0</v>
@@ -58185,8 +58205,8 @@
       <c r="DO52">
         <v>0</v>
       </c>
-      <c r="DP52">
-        <v>0</v>
+      <c r="DP52" s="2">
+        <v>1</v>
       </c>
       <c r="DQ52">
         <v>0</v>
@@ -58293,8 +58313,8 @@
       <c r="EY52">
         <v>0</v>
       </c>
-      <c r="EZ52">
-        <v>0</v>
+      <c r="EZ52" s="2">
+        <v>1</v>
       </c>
       <c r="FA52">
         <v>0</v>
@@ -58425,8 +58445,8 @@
       <c r="GQ52">
         <v>0</v>
       </c>
-      <c r="GR52">
-        <v>0</v>
+      <c r="GR52" s="2">
+        <v>1</v>
       </c>
       <c r="GS52">
         <v>0</v>
@@ -58593,8 +58613,8 @@
       <c r="IU52">
         <v>0</v>
       </c>
-      <c r="IV52">
-        <v>0</v>
+      <c r="IV52" s="2">
+        <v>1</v>
       </c>
       <c r="IW52">
         <v>0</v>
@@ -59207,8 +59227,8 @@
       <c r="CR53">
         <v>0</v>
       </c>
-      <c r="CS53">
-        <v>0</v>
+      <c r="CS53" s="2">
+        <v>1</v>
       </c>
       <c r="CT53">
         <v>0</v>
@@ -60298,8 +60318,8 @@
       <c r="CR54">
         <v>0</v>
       </c>
-      <c r="CS54">
-        <v>0</v>
+      <c r="CS54" s="2">
+        <v>1</v>
       </c>
       <c r="CT54">
         <v>0</v>
@@ -60331,20 +60351,20 @@
       <c r="DC54">
         <v>0</v>
       </c>
-      <c r="DD54">
-        <v>0</v>
+      <c r="DD54" s="2">
+        <v>1</v>
       </c>
       <c r="DE54">
         <v>0</v>
       </c>
-      <c r="DF54">
-        <v>0</v>
-      </c>
-      <c r="DG54">
-        <v>0</v>
-      </c>
-      <c r="DH54">
-        <v>0</v>
+      <c r="DF54" s="2">
+        <v>1</v>
+      </c>
+      <c r="DG54" s="2">
+        <v>1</v>
+      </c>
+      <c r="DH54" s="2">
+        <v>1</v>
       </c>
       <c r="DI54">
         <v>0</v>
@@ -60367,8 +60387,8 @@
       <c r="DO54">
         <v>0</v>
       </c>
-      <c r="DP54">
-        <v>0</v>
+      <c r="DP54" s="2">
+        <v>1</v>
       </c>
       <c r="DQ54">
         <v>0</v>
@@ -60475,8 +60495,8 @@
       <c r="EY54">
         <v>0</v>
       </c>
-      <c r="EZ54">
-        <v>0</v>
+      <c r="EZ54" s="2">
+        <v>1</v>
       </c>
       <c r="FA54">
         <v>0</v>
@@ -60511,8 +60531,8 @@
       <c r="FK54">
         <v>0</v>
       </c>
-      <c r="FL54">
-        <v>0</v>
+      <c r="FL54" s="2">
+        <v>1</v>
       </c>
       <c r="FM54">
         <v>0</v>
@@ -60520,8 +60540,8 @@
       <c r="FN54">
         <v>0</v>
       </c>
-      <c r="FO54">
-        <v>0</v>
+      <c r="FO54" s="2">
+        <v>1</v>
       </c>
       <c r="FP54">
         <v>0</v>
@@ -60529,14 +60549,14 @@
       <c r="FQ54">
         <v>0</v>
       </c>
-      <c r="FR54">
-        <v>0</v>
+      <c r="FR54" s="2">
+        <v>1</v>
       </c>
       <c r="FS54">
         <v>0</v>
       </c>
-      <c r="FT54">
-        <v>0</v>
+      <c r="FT54" s="2">
+        <v>1</v>
       </c>
       <c r="FU54">
         <v>0</v>
@@ -60625,8 +60645,8 @@
       <c r="GW54">
         <v>0</v>
       </c>
-      <c r="GX54">
-        <v>0</v>
+      <c r="GX54" s="2">
+        <v>1</v>
       </c>
       <c r="GY54">
         <v>0</v>
@@ -60727,8 +60747,8 @@
       <c r="IE54">
         <v>0</v>
       </c>
-      <c r="IF54">
-        <v>0</v>
+      <c r="IF54" s="2">
+        <v>1</v>
       </c>
       <c r="IG54">
         <v>0</v>
@@ -60991,8 +61011,8 @@
       <c r="LO54">
         <v>0</v>
       </c>
-      <c r="LP54">
-        <v>0</v>
+      <c r="LP54" s="2">
+        <v>1</v>
       </c>
       <c r="LQ54">
         <v>0</v>
@@ -61389,8 +61409,8 @@
       <c r="CR55">
         <v>0</v>
       </c>
-      <c r="CS55">
-        <v>0</v>
+      <c r="CS55" s="2">
+        <v>1</v>
       </c>
       <c r="CT55">
         <v>0</v>
@@ -61413,8 +61433,8 @@
       <c r="CZ55">
         <v>0</v>
       </c>
-      <c r="DA55">
-        <v>0</v>
+      <c r="DA55" s="2">
+        <v>1</v>
       </c>
       <c r="DB55">
         <v>0</v>
@@ -61422,8 +61442,8 @@
       <c r="DC55">
         <v>0</v>
       </c>
-      <c r="DD55">
-        <v>0</v>
+      <c r="DD55" s="2">
+        <v>1</v>
       </c>
       <c r="DE55">
         <v>0</v>
@@ -61431,8 +61451,8 @@
       <c r="DF55">
         <v>0</v>
       </c>
-      <c r="DG55">
-        <v>0</v>
+      <c r="DG55" s="2">
+        <v>1</v>
       </c>
       <c r="DH55">
         <v>0</v>
@@ -61458,8 +61478,8 @@
       <c r="DO55">
         <v>0</v>
       </c>
-      <c r="DP55">
-        <v>0</v>
+      <c r="DP55" s="2">
+        <v>1</v>
       </c>
       <c r="DQ55">
         <v>0</v>
@@ -61602,8 +61622,8 @@
       <c r="FK55">
         <v>0</v>
       </c>
-      <c r="FL55">
-        <v>0</v>
+      <c r="FL55" s="2">
+        <v>1</v>
       </c>
       <c r="FM55">
         <v>0</v>
@@ -61626,8 +61646,8 @@
       <c r="FS55">
         <v>0</v>
       </c>
-      <c r="FT55">
-        <v>0</v>
+      <c r="FT55" s="2">
+        <v>1</v>
       </c>
       <c r="FU55">
         <v>0</v>
@@ -61641,8 +61661,8 @@
       <c r="FX55">
         <v>0</v>
       </c>
-      <c r="FY55">
-        <v>0</v>
+      <c r="FY55" s="2">
+        <v>1</v>
       </c>
       <c r="FZ55">
         <v>0</v>
@@ -61704,8 +61724,8 @@
       <c r="GS55">
         <v>1</v>
       </c>
-      <c r="GT55">
-        <v>0</v>
+      <c r="GT55" s="2">
+        <v>1</v>
       </c>
       <c r="GU55">
         <v>0</v>
@@ -61818,8 +61838,8 @@
       <c r="IE55">
         <v>0</v>
       </c>
-      <c r="IF55">
-        <v>0</v>
+      <c r="IF55" s="2">
+        <v>1</v>
       </c>
       <c r="IG55">
         <v>0</v>
@@ -61845,8 +61865,8 @@
       <c r="IN55">
         <v>0</v>
       </c>
-      <c r="IO55">
-        <v>0</v>
+      <c r="IO55" s="2">
+        <v>1</v>
       </c>
       <c r="IP55">
         <v>0</v>
@@ -61866,8 +61886,8 @@
       <c r="IU55">
         <v>0</v>
       </c>
-      <c r="IV55">
-        <v>0</v>
+      <c r="IV55" s="2">
+        <v>1</v>
       </c>
       <c r="IW55">
         <v>0</v>
@@ -61875,8 +61895,8 @@
       <c r="IX55">
         <v>0</v>
       </c>
-      <c r="IY55">
-        <v>0</v>
+      <c r="IY55" s="2">
+        <v>1</v>
       </c>
       <c r="IZ55">
         <v>0</v>
@@ -62462,8 +62482,8 @@
       <c r="CL56">
         <v>0</v>
       </c>
-      <c r="CM56">
-        <v>0</v>
+      <c r="CM56" s="2">
+        <v>1</v>
       </c>
       <c r="CN56">
         <v>0</v>
@@ -63571,8 +63591,8 @@
       <c r="CR57">
         <v>0</v>
       </c>
-      <c r="CS57">
-        <v>0</v>
+      <c r="CS57" s="2">
+        <v>1</v>
       </c>
       <c r="CT57">
         <v>0</v>
@@ -63640,8 +63660,8 @@
       <c r="DO57">
         <v>0</v>
       </c>
-      <c r="DP57">
-        <v>0</v>
+      <c r="DP57" s="2">
+        <v>1</v>
       </c>
       <c r="DQ57">
         <v>0</v>
@@ -64695,8 +64715,8 @@
       <c r="DC58">
         <v>0</v>
       </c>
-      <c r="DD58">
-        <v>0</v>
+      <c r="DD58" s="2">
+        <v>1</v>
       </c>
       <c r="DE58">
         <v>0</v>
@@ -64704,8 +64724,8 @@
       <c r="DF58">
         <v>0</v>
       </c>
-      <c r="DG58">
-        <v>0</v>
+      <c r="DG58" s="2">
+        <v>1</v>
       </c>
       <c r="DH58">
         <v>0</v>
@@ -64971,8 +64991,8 @@
       <c r="GQ58">
         <v>0</v>
       </c>
-      <c r="GR58">
-        <v>0</v>
+      <c r="GR58" s="2">
+        <v>1</v>
       </c>
       <c r="GS58">
         <v>0</v>
@@ -69206,8 +69226,8 @@
       <c r="EZ62">
         <v>0</v>
       </c>
-      <c r="FA62">
-        <v>0</v>
+      <c r="FA62" s="2">
+        <v>1</v>
       </c>
       <c r="FB62">
         <v>0</v>
@@ -69455,8 +69475,8 @@
       <c r="IE62">
         <v>0</v>
       </c>
-      <c r="IF62">
-        <v>0</v>
+      <c r="IF62" s="2">
+        <v>1</v>
       </c>
       <c r="IG62">
         <v>0</v>
@@ -70081,8 +70101,8 @@
       <c r="CF63">
         <v>0</v>
       </c>
-      <c r="CG63">
-        <v>0</v>
+      <c r="CG63" s="2">
+        <v>1</v>
       </c>
       <c r="CH63">
         <v>0</v>
@@ -70123,8 +70143,8 @@
       <c r="CT63">
         <v>0</v>
       </c>
-      <c r="CU63">
-        <v>0</v>
+      <c r="CU63" s="2">
+        <v>1</v>
       </c>
       <c r="CV63">
         <v>0</v>
@@ -70141,8 +70161,8 @@
       <c r="CZ63">
         <v>0</v>
       </c>
-      <c r="DA63">
-        <v>0</v>
+      <c r="DA63" s="2">
+        <v>1</v>
       </c>
       <c r="DB63">
         <v>0</v>
@@ -70157,7 +70177,7 @@
         <v>0</v>
       </c>
       <c r="DF63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DG63">
         <v>0</v>
@@ -70294,11 +70314,11 @@
       <c r="EY63">
         <v>0</v>
       </c>
-      <c r="EZ63">
-        <v>0</v>
-      </c>
-      <c r="FA63">
-        <v>0</v>
+      <c r="EZ63" s="2">
+        <v>1</v>
+      </c>
+      <c r="FA63" s="2">
+        <v>1</v>
       </c>
       <c r="FB63">
         <v>0</v>
@@ -70348,8 +70368,8 @@
       <c r="FQ63">
         <v>0</v>
       </c>
-      <c r="FR63">
-        <v>0</v>
+      <c r="FR63" s="2">
+        <v>1</v>
       </c>
       <c r="FS63">
         <v>0</v>
@@ -70600,8 +70620,8 @@
       <c r="IW63">
         <v>0</v>
       </c>
-      <c r="IX63">
-        <v>0</v>
+      <c r="IX63" s="2">
+        <v>1</v>
       </c>
       <c r="IY63">
         <v>0</v>
@@ -70612,8 +70632,8 @@
       <c r="JA63">
         <v>0</v>
       </c>
-      <c r="JB63">
-        <v>0</v>
+      <c r="JB63" s="2">
+        <v>1</v>
       </c>
       <c r="JC63">
         <v>1</v>
@@ -76387,8 +76407,8 @@
       <c r="D69">
         <v>0</v>
       </c>
-      <c r="E69">
-        <v>0</v>
+      <c r="E69" s="2">
+        <v>1</v>
       </c>
       <c r="F69">
         <v>1</v>
@@ -76408,8 +76428,8 @@
       <c r="K69">
         <v>0</v>
       </c>
-      <c r="L69">
-        <v>0</v>
+      <c r="L69" s="2">
+        <v>1</v>
       </c>
       <c r="M69">
         <v>0</v>
@@ -76627,8 +76647,8 @@
       <c r="CF69">
         <v>0</v>
       </c>
-      <c r="CG69">
-        <v>0</v>
+      <c r="CG69" s="2">
+        <v>1</v>
       </c>
       <c r="CH69">
         <v>0</v>
@@ -76687,14 +76707,14 @@
       <c r="CZ69">
         <v>0</v>
       </c>
-      <c r="DA69">
-        <v>0</v>
+      <c r="DA69" s="2">
+        <v>1</v>
       </c>
       <c r="DB69">
         <v>0</v>
       </c>
-      <c r="DC69">
-        <v>0</v>
+      <c r="DC69" s="2">
+        <v>1</v>
       </c>
       <c r="DD69">
         <v>0</v>
@@ -76702,8 +76722,8 @@
       <c r="DE69">
         <v>0</v>
       </c>
-      <c r="DF69">
-        <v>0</v>
+      <c r="DF69" s="2">
+        <v>1</v>
       </c>
       <c r="DG69">
         <v>1</v>
@@ -76840,8 +76860,8 @@
       <c r="EY69">
         <v>0</v>
       </c>
-      <c r="EZ69">
-        <v>0</v>
+      <c r="EZ69" s="2">
+        <v>1</v>
       </c>
       <c r="FA69">
         <v>1</v>
@@ -76852,8 +76872,8 @@
       <c r="FC69">
         <v>0</v>
       </c>
-      <c r="FD69">
-        <v>0</v>
+      <c r="FD69" s="2">
+        <v>1</v>
       </c>
       <c r="FE69">
         <v>0</v>
@@ -76876,8 +76896,8 @@
       <c r="FK69">
         <v>0</v>
       </c>
-      <c r="FL69">
-        <v>0</v>
+      <c r="FL69" s="2">
+        <v>1</v>
       </c>
       <c r="FM69">
         <v>0</v>
@@ -76900,8 +76920,8 @@
       <c r="FS69">
         <v>0</v>
       </c>
-      <c r="FT69">
-        <v>0</v>
+      <c r="FT69" s="2">
+        <v>1</v>
       </c>
       <c r="FU69">
         <v>0</v>
@@ -76954,8 +76974,8 @@
       <c r="GK69">
         <v>0</v>
       </c>
-      <c r="GL69">
-        <v>0</v>
+      <c r="GL69" s="2">
+        <v>1</v>
       </c>
       <c r="GM69">
         <v>0</v>
@@ -77119,8 +77139,8 @@
       <c r="IN69">
         <v>0</v>
       </c>
-      <c r="IO69">
-        <v>0</v>
+      <c r="IO69" s="2">
+        <v>1</v>
       </c>
       <c r="IP69">
         <v>0</v>
@@ -77158,11 +77178,11 @@
       <c r="JA69">
         <v>0</v>
       </c>
-      <c r="JB69">
-        <v>0</v>
-      </c>
-      <c r="JC69">
-        <v>0</v>
+      <c r="JB69" s="2">
+        <v>1</v>
+      </c>
+      <c r="JC69" s="2">
+        <v>1</v>
       </c>
       <c r="JD69">
         <v>0</v>
@@ -77793,8 +77813,8 @@
       <c r="DE70">
         <v>0</v>
       </c>
-      <c r="DF70">
-        <v>0</v>
+      <c r="DF70" s="2">
+        <v>1</v>
       </c>
       <c r="DG70">
         <v>0</v>
@@ -78525,8 +78545,8 @@
       <c r="MO70">
         <v>0</v>
       </c>
-      <c r="MP70">
-        <v>0</v>
+      <c r="MP70" s="2">
+        <v>1</v>
       </c>
       <c r="MQ70">
         <v>0</v>
@@ -78845,8 +78865,8 @@
       <c r="CR71">
         <v>0</v>
       </c>
-      <c r="CS71">
-        <v>0</v>
+      <c r="CS71" s="2">
+        <v>1</v>
       </c>
       <c r="CT71">
         <v>0</v>
@@ -78902,8 +78922,8 @@
       <c r="DK71">
         <v>0</v>
       </c>
-      <c r="DL71">
-        <v>0</v>
+      <c r="DL71" s="2">
+        <v>1</v>
       </c>
       <c r="DM71">
         <v>0</v>
@@ -79058,8 +79078,8 @@
       <c r="FK71">
         <v>0</v>
       </c>
-      <c r="FL71">
-        <v>0</v>
+      <c r="FL71" s="2">
+        <v>1</v>
       </c>
       <c r="FM71">
         <v>0</v>
@@ -79067,8 +79087,8 @@
       <c r="FN71">
         <v>0</v>
       </c>
-      <c r="FO71">
-        <v>0</v>
+      <c r="FO71" s="2">
+        <v>1</v>
       </c>
       <c r="FP71">
         <v>0</v>
@@ -79076,14 +79096,14 @@
       <c r="FQ71">
         <v>0</v>
       </c>
-      <c r="FR71">
-        <v>0</v>
+      <c r="FR71" s="2">
+        <v>1</v>
       </c>
       <c r="FS71">
         <v>0</v>
       </c>
-      <c r="FT71">
-        <v>0</v>
+      <c r="FT71" s="2">
+        <v>1</v>
       </c>
       <c r="FU71">
         <v>0</v>
@@ -79211,8 +79231,8 @@
       <c r="HJ71">
         <v>0</v>
       </c>
-      <c r="HK71">
-        <v>0</v>
+      <c r="HK71" s="2">
+        <v>1</v>
       </c>
       <c r="HL71">
         <v>0</v>
@@ -79274,8 +79294,8 @@
       <c r="IE71">
         <v>0</v>
       </c>
-      <c r="IF71">
-        <v>0</v>
+      <c r="IF71" s="2">
+        <v>1</v>
       </c>
       <c r="IG71">
         <v>0</v>
@@ -79771,8 +79791,8 @@
       <c r="AO72">
         <v>0</v>
       </c>
-      <c r="AP72">
-        <v>0</v>
+      <c r="AP72" s="2">
+        <v>1</v>
       </c>
       <c r="AQ72">
         <v>0</v>
@@ -79915,8 +79935,8 @@
       <c r="CK72">
         <v>0</v>
       </c>
-      <c r="CL72">
-        <v>0</v>
+      <c r="CL72" s="2">
+        <v>1</v>
       </c>
       <c r="CM72">
         <v>0</v>
@@ -79960,17 +79980,26 @@
       <c r="CZ72">
         <v>0</v>
       </c>
+      <c r="DA72" s="2">
+        <v>1</v>
+      </c>
+      <c r="DB72">
+        <v>0</v>
+      </c>
+      <c r="DC72">
+        <v>0</v>
+      </c>
       <c r="DD72">
         <v>0</v>
       </c>
       <c r="DE72">
         <v>0</v>
       </c>
-      <c r="DF72">
-        <v>0</v>
-      </c>
-      <c r="DG72">
-        <v>0</v>
+      <c r="DF72" s="2">
+        <v>1</v>
+      </c>
+      <c r="DG72" s="2">
+        <v>1</v>
       </c>
       <c r="DH72">
         <v>0</v>
@@ -79996,8 +80025,8 @@
       <c r="DO72">
         <v>0</v>
       </c>
-      <c r="DP72">
-        <v>0</v>
+      <c r="DP72" s="2">
+        <v>1</v>
       </c>
       <c r="DQ72">
         <v>0</v>
@@ -80107,8 +80136,8 @@
       <c r="EZ72">
         <v>0</v>
       </c>
-      <c r="FA72">
-        <v>0</v>
+      <c r="FA72" s="2">
+        <v>1</v>
       </c>
       <c r="FB72">
         <v>0</v>
@@ -80164,8 +80193,8 @@
       <c r="FS72">
         <v>0</v>
       </c>
-      <c r="FT72">
-        <v>0</v>
+      <c r="FT72" s="2">
+        <v>1</v>
       </c>
       <c r="FU72">
         <v>0</v>
@@ -80188,6 +80217,9 @@
       <c r="GA72">
         <v>0</v>
       </c>
+      <c r="GB72">
+        <v>0</v>
+      </c>
       <c r="GC72">
         <v>0</v>
       </c>
@@ -80215,8 +80247,8 @@
       <c r="GK72">
         <v>0</v>
       </c>
-      <c r="GL72">
-        <v>0</v>
+      <c r="GL72" s="2">
+        <v>1</v>
       </c>
       <c r="GM72">
         <v>0</v>
@@ -80380,8 +80412,8 @@
       <c r="IN72">
         <v>0</v>
       </c>
-      <c r="IO72">
-        <v>0</v>
+      <c r="IO72" s="2">
+        <v>1</v>
       </c>
       <c r="IP72">
         <v>0</v>
@@ -80407,8 +80439,8 @@
       <c r="IW72">
         <v>0</v>
       </c>
-      <c r="IX72">
-        <v>0</v>
+      <c r="IX72" s="2">
+        <v>1</v>
       </c>
       <c r="IY72">
         <v>0</v>
@@ -80566,8 +80598,8 @@
       <c r="KX72">
         <v>0</v>
       </c>
-      <c r="KY72">
-        <v>0</v>
+      <c r="KY72" s="2">
+        <v>1</v>
       </c>
       <c r="KZ72">
         <v>0</v>
@@ -80695,8 +80727,8 @@
       <c r="MO72">
         <v>0</v>
       </c>
-      <c r="MP72">
-        <v>0</v>
+      <c r="MP72" s="2">
+        <v>1</v>
       </c>
       <c r="MQ72">
         <v>0</v>
@@ -80722,8 +80754,8 @@
       <c r="MX72">
         <v>0</v>
       </c>
-      <c r="MY72">
-        <v>0</v>
+      <c r="MY72" s="2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>